<commit_message>
Leads: 2026-09-23 00:05 UTC (cycle 182)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scottsdale Roofing Contractor - 30+ Yrs in AZ | Free Estimate | Paragon</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>paragonbuiltaz.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.paragonbuiltaz.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>System Plus</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>info@paragonbuiltaz.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(928) 237-2955</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Scottsdale AZ</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>88</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>roofing contractor Scottsdale AZ</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 00:09 UTC (cycle 185)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SOS Water Heater Pearland</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pearland.soswaterheater.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://pearland.soswaterheater.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Heater Pearland</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>service@houston.soswaterheater.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>346-569-8172</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pearland TX</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>94</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>water heater repair Pearland TX</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 00:11 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hometown Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>hometownroofing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://hometownroofing.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Council Bluffs</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@hometownroofing.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>402-896-3639</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofer Omaha NE</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 00:12 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>New Pipes Inc.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>newpipesinc.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.newpipesinc.com/plumbing/plumbing-company-fremont-ca/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>connect@solutionarian.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(408) 269-1969</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>plumbing company Fremont CA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 00:17 UTC (cycle 190)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -803,6 +803,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HVAC Contractor in Broken Arrow, OK</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>rescueheatandair.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://rescueheatandair.com/service-areas/broken-arrow-ok-hvac-services/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Solutions Given</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ronak.patel@esplindia.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>918-946-6681</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HVAC contractor Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 00:20 UTC (cycle 192)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -863,6 +863,62 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HVAC Repair in Dover, DE — 4.8★ Rated | Same-Day Service</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>jemcomfortcare.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://jemcomfortcare.com/hvac-dover-de/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>jemcomfortcare@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>302-515-0777</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Dover DE</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>furnace repair Dover DE</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 00:33 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -884,7 +884,6 @@
           <t>https://jemcomfortcare.com/hvac-dover-de/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>jemcomfortcare@gmail.com</t>
@@ -914,6 +913,66 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HS Drain</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hsdrainsnys.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://hsdrainsnys.com/services/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Plumbing Professionals</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>hsdrainsnys@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(914) 227-8996</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Yonkers NY</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>84</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>drain cleaning service Yonkers NY</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 00:34 UTC (cycle 202)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Super Service Today</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>superservicetoday.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://superservicetoday.com/services/drain-sewer/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Pack When</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>superservicetoday@gmail.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(781) 519-9921</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>drain cleaning service Boston MA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:30 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1038,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Expert HVAC Contractors - Reno, NV - Precision Air</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>precisionairnv.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.precisionairnv.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Precision Air</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>jledkins1@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(775) 481-5079</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Reno NV</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>HVAC contractor Reno NV</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:36 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,62 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bright Star Service</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>brightstarservice.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://brightstarservice.com/furnace-repair-new-york-city/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@brightstarservice.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(212) 516-9632</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>New York NY</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>84</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>furnace repair New York NY</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:38 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1119,7 +1119,6 @@
           <t>https://brightstarservice.com/furnace-repair-new-york-city/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>info@brightstarservice.com</t>
@@ -1149,6 +1148,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Affordable Home A/C</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>affordablehome-ac.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.affordablehome-ac.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Verified Reviews</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>office@affordablehome-ac.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(808) 488-1111</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>84</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>AC installation Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:39 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1213,6 +1213,58 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Roofer Iowa City, IA | Martinez Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>martinezroofingia.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.martinezroofingia.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>jmartinezroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Iowa City IA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>76</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roof replacement Iowa City IA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:41 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1234,13 +1234,11 @@
           <t>https://www.martinezroofingia.com/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>jmartinezroofing@gmail.com</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Iowa City IA</t>
@@ -1260,6 +1258,62 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair Services | Orlando, FL | Dial Septic Tank Service Inc.</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>dialseptic.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.dialseptic.com/sewer-line-repair-services/orlando-fl</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>eliie@dialseptic.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>407-365-4549</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>92</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>sewer repair Orlando FL</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:42 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1284,7 +1284,6 @@
           <t>https://www.dialseptic.com/sewer-line-repair-services/orlando-fl</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>eliie@dialseptic.com</t>
@@ -1314,6 +1313,118 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair | Missoula County MT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>rotorootermissoula.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.rotorootermissoula.com/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>modanhalstead@aol.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(406) 344-4477</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Missoula MT</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>sewer repair Missoula MT</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Acadiana Plumbing</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>acadianaplumbing.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://acadianaplumbing.com/water-heater-1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>team@latofonts.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(337) 703-3939</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>84</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>water heater repair Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:45 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1339,7 +1339,6 @@
           <t>https://www.rotorootermissoula.com/sewer-line-repair</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>modanhalstead@aol.com</t>
@@ -1395,7 +1394,6 @@
           <t>https://acadianaplumbing.com/water-heater-1</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>team@latofonts.com</t>
@@ -1425,6 +1423,66 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Roof Replacement | Columbus, GA | Danny Renfroe's Roofing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dannyrenfroesroofing.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.dannyrenfroesroofing.com/roof-replacement-columbus-ga</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Danny Renfroe</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>shanerenfroe44@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(706)-568-6626</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Columbus GA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roof replacement Columbus GA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:54 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1488,6 +1488,62 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Dayton Roofing</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>daytonroofing.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.daytonroofing.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>allen@daytonroofing.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(937) 829-9500</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Dayton OH</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>88</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>roof replacement Dayton OH</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 13:55 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1509,7 +1509,6 @@
           <t>https://www.daytonroofing.com/</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>allen@daytonroofing.com</t>
@@ -1539,6 +1538,62 @@
         </is>
       </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Authentic Roofing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>authenticroofing.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.authenticroofing.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>mary@authenticroofing.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>775.560.1450</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Sparks NV</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>residential roofing company Sparks NV</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 14:13 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1564,7 +1564,6 @@
           <t>https://www.authenticroofing.com/</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>mary@authenticroofing.com</t>
@@ -1594,6 +1593,66 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>New Braunfels Roof Repair &amp; Replacement | Lunar Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>lunarroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://lunarroofingtx.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Lunar Roofing</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>office@lunarroofingtx.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>830-800-0252</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roof replacement New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 14:15 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1658,6 +1658,66 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rival Digital Boilerplate</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>samedayhvacservices.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://samedayhvacservices.com/air-conditioning/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Same Day</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>samedayhvacservices@gmail.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>510-887-5571</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>air conditioning repair San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 14:37 UTC (cycle 46)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1718,6 +1718,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Metal Roofing Contractors | Metal Roofing Installation &amp; Repair</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>fortifiedroofs.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.fortifiedroofs.com/roofing/metal/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No Reviews</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>hello@fortifiedroofs.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(573) 269-3845</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Columbia MO</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Columbia MO</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 14:40 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1778,6 +1778,66 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Non-Stop Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>nonstopair-fl.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.nonstopair-fl.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Cape Coral</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>support@nonstopair-fl.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>239-990-5399</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>HVAC contractor Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 14:41 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1838,6 +1838,118 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair — Hoffman Plumbing Pittsburgh</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>hoffmanplumbingpgh.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://hoffmanplumbingpgh.com/services/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>info@hoffmanplumbingpittsburgh.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>412-265-5479</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>sewer repair Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Trenchless Sewer Repair | Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>brickhaas.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.brickhaas.com/trenchless-sewer-repair</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>brickhaasplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(412) 206-1868</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>sewer repair Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 14:43 UTC (cycle 50)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1859,7 +1859,6 @@
           <t>https://hoffmanplumbingpgh.com/services/sewer-line-repair</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>info@hoffmanplumbingpittsburgh.com</t>
@@ -1915,7 +1914,6 @@
           <t>https://www.brickhaas.com/trenchless-sewer-repair</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>brickhaasplumbing@gmail.com</t>
@@ -1945,6 +1943,118 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tampa Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>tampa-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://tampa-metal-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>info@tampa-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(656) 235-2584</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Tampa FL</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Hytz Roofing</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>hytzroofing.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://hytzroofing.com/metal-roofing-tampa</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>office@hytzroofing.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(813) 436-0761</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>76</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Tampa FL</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 14:55 UTC (cycle 58)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1969,7 +1969,6 @@
           <t>https://tampa-metal-roofing.com/</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>info@tampa-metal-roofing.com</t>
@@ -2025,7 +2024,6 @@
           <t>https://hytzroofing.com/metal-roofing-tampa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>office@hytzroofing.com</t>
@@ -2055,6 +2053,66 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Concord Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>concordroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://concordroofingtx.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>What Our</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>info@concordroofingtx.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(214) 299-6110</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>90</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>roofing contractor Plano TX</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 15:00 UTC (cycle 62)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2118,6 +2118,66 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Greeley Roofer</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>gusroofing.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.gusroofing.com/cheyenne-wy-roofing-company/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Inspections Our</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>gusroofing@gusroofing.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>970-356-1554</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>90</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>roofing contractor Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 15:02 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2178,6 +2178,66 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Guthrie Plumbing &amp; H</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>guthrieplumbingandheating.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.guthrieplumbingandheating.com/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Owners Michelle</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>guthrieplumbing.dale@gmail.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>218-727-8733</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>100</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>plumbing company Duluth MN</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 15:14 UTC (cycle 71)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2238,6 +2238,66 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Heat Pump Install Conroe, TX | Heat Pump Service</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>vaneddies.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.vaneddies.com/heat-pump/heat-pump-installation-conroe-tx</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Conroe Homeowners</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>office@vaneddie.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(321) 663-2665</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>heat pump installation Conroe TX</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 15:29 UTC (cycle 81)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2298,6 +2298,66 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>White &amp; Sons Roofing</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>whiteandsonsroofingpa.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://whiteandsonsroofingpa.com/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sons Roofing</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>whiteandsonsrfg@gmail.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(610) 914-5115</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Reading PA</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>roof replacement Reading PA</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 15:31 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2358,6 +2358,66 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>John’s Heating, Cooling, and Plumbing</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>justcalljohns.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.justcalljohns.com/hvac-repair-replacement-scottsdale-az</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Andrew John</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>dsgorm@netzero.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>480.649.1000</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Scottsdale AZ</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>90</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>furnace repair Scottsdale AZ</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 15:34 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2418,6 +2418,122 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Magnolia Air Solutions</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>magnoliaairsolutions.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.magnoliaairsolutions.com/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Magnolia Air</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>kirstie@magnoliaairsolutions.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(251) 486-2026</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Mobile AL</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>100</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>AC installation Mobile AL</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>AC Installation | Mobile, AL | T. Batchelor and Son</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>tbatchelorandson.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.tbatchelorandson.com/heating-cooling-installation-mobile-al</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>dbatchelor@tbatchelorandson.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>251-250-1291</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Mobile AL</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>88</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>AC installation Mobile AL</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 15:38 UTC (cycle 87)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2499,7 +2499,6 @@
           <t>https://www.tbatchelorandson.com/heating-cooling-installation-mobile-al</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>dbatchelor@tbatchelorandson.com</t>
@@ -2529,6 +2528,66 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Logams Roofing</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>logamsroofing.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.logamsroofing.com/roofing-company-ocala</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Counties Orange</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>info@logamsroofing.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>321-386-1794</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>residential roofing company Ocala FL</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 15:50 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2593,6 +2593,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Expert Air Conditioning Services for Oahu and Big Island | Your Trusted HVAC Con</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>craigsair.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.craigsair.com/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Kevin Mederos</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>service@craigsair.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(808) 682-0970</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>88</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>HVAC contractor Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 16:03 UTC (cycle 104)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2653,6 +2653,66 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Durham Roofing Company | Pickard Roofing</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>pickardroofing.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.pickardroofing.com/durham-roofing-company</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Family James</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@pickardroofing.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>919-682-5702</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>90</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>roofer Durham NC</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 16:09 UTC (cycle 108)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2713,6 +2713,66 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Top-Notch Metal Roofing in Scranton</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>bittnerroofs.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://bittnerroofs.com/metal-roofing-scranton/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>What Homeowners</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>info@nepahomepros.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>570-241-3500</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Scranton PA</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>100</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Scranton PA</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 16:18 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2773,6 +2773,62 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Anubis Mechanical, LLC</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>anubismechanical.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://anubismechanical.com/residential/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>noreply@anubismechanical.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>(843) 343-8753</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>North Charleston SC</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>90</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>heat pump installation North Charleston SC</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 16:24 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2794,7 +2794,6 @@
           <t>https://anubismechanical.com/residential/heat-pumps/</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>noreply@anubismechanical.com</t>
@@ -2824,6 +2823,66 @@
         </is>
       </c>
       <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Cleveland Plumber</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>clevelandsplumber.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://clevelandsplumber.com/serving-areas/parma</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>On The</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>service@clevelandsplumber.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(216) 595-0793</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Parma OH</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>drain cleaning service Parma OH</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 16:33 UTC (cycle 124)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2888,6 +2888,66 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>A&amp;K Service Inc.</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>akservice-hvac.org</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://akservice-hvac.org/areas/sandy-springs-ga</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Service Inc</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>akservicehvac1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(770) 475-0628</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>100</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>HVAC contractor Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 16:40 UTC (cycle 129)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2948,6 +2948,126 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Gorillaroofingpros</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>gorillaroofingpros.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.gorillaroofingpros.com/roofing-lowell-ma</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>New Hampshire</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>sales@gorillaroofingpros.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>978-737-7320</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Lowell MA</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>96</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>roof replacement Lowell MA</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Ann Arbor</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>southfieldroofingpros.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.southfieldroofingpros.com/locations/ann-arbor-mi/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Angell Eberwhite</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>info@southfieldroofingpros.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>(877) 657-4792</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>90</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 16:43 UTC (cycle 131)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3068,6 +3068,122 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>My Vxw Site Y2tcjr</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>hickory-roofing.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.hickory-roofing.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(717)321-4058</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>York PA</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>100</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>metal roofing contractor York PA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Boise Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>boise-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://boise-metal-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>info@boise-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(208) 900-4692</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>100</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Boise ID</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 16:46 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3089,7 +3089,6 @@
           <t>https://www.hickory-roofing.com/metal-roofing</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>example@mysite.com</t>
@@ -3179,6 +3178,122 @@
         </is>
       </c>
       <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Plumber Elite of Utica</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>plumberelitetheutica.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://plumberelitetheutica.com/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Services Our</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>info@plumbereliteutica.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>(315) 750-3284</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Utica NY</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>90</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>plumbing company Utica NY</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>A&amp;R Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>aandrplumbingcny.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://aandrplumbingcny.com/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>aandrplumbingcny@gmail.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>315-768-6668</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Utica NY</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>84</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>plumbing company Utica NY</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 17:02 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3264,7 +3264,6 @@
           <t>https://aandrplumbingcny.com/</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>aandrplumbingcny@gmail.com</t>
@@ -3294,6 +3293,62 @@
         </is>
       </c>
       <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Phoenix, Arizona Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>stradroofing.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://stradroofing.com/phoenix-roofer/stradling-roofing-locations/gilbert-arizona-roofing-contractor/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>info@stradroofing.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(480) 901-6901</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>98</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>roof repair company Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 17:06 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3319,7 +3319,6 @@
           <t>https://stradroofing.com/phoenix-roofer/stradling-roofing-locations/gilbert-arizona-roofing-contractor/</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>info@stradroofing.com</t>
@@ -3349,6 +3348,66 @@
         </is>
       </c>
       <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Max Chill Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>hialeahflacrepair.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.hialeahflacrepair.com/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Max Chill</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>info@hialeahflacrepair.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(645) 230-0400</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>90</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>heating and cooling company Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 17:11 UTC (cycle 150)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3413,6 +3413,66 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>KPro Roofing &amp; Renovation</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>go2kpro.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://go2kpro.com/locations-ofallon</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Founder Kyle</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>info@go2kpro.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(636) 557-5919</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>OFallon MO</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>roofing contractor OFallon MO</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 17:17 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3473,6 +3473,66 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Water Heater Oakland | Repair &amp; Install | Z and Z Plumbing</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>zandzplumbing.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.zandzplumbing.com/water-heater-oakland/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Team One</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>info@zandzplumbing.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(510) 708-4237</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Oakland CA</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>90</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>water heater repair Oakland CA</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 17:24 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3533,6 +3533,122 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>HVAC Company Missouri</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ac-installation-lees-summit.heatingcoolingmacon.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://ac-installation-lees-summit.heatingcoolingmacon.com/</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Lees Summit</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>admin@sood.heritageplumbinggrantspass.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(888) 709-2550</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>100</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>AC installation Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Floyd's Plumbing</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>floydsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://floydsplumbing.com/services/water-heaters/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>kenny@floydtheplumber.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(352) 304-6404</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>90</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>water heater repair Ocala FL</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 17:39 UTC (cycle 169)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3614,7 +3614,6 @@
           <t>https://floydsplumbing.com/services/water-heaters/</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>kenny@floydtheplumber.com</t>
@@ -3644,6 +3643,66 @@
         </is>
       </c>
       <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Samuel Roofing</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>samuelroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://samuelroofinginc.com/irvine-roofing/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>samuelroofinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(866) 685-3889</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>roof replacement Irvine CA</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 17:42 UTC (cycle 171)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3708,6 +3708,126 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Water Heater Services Plymouth, MN</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>knightsplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://knightsplumbingllc.com/areas-of-service/water-heater-services-plymouth/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Knights Plumbing</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>info@knightsplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>(763) 286-9941</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Plymouth MN</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>100</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>water heater repair Plymouth MN</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Excavation &amp; Sewer Services | Z.R. Russell LLC | Harrisburg</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>zrrussell.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://zrrussell.com/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Zachary Russell</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>zrrussell87@gmail.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(717) 421-1895</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>84</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>sewer repair Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 18:06 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3828,6 +3828,62 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Metal Roof Charleston</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>metalroofcharleston.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://www.metalroofcharleston.com/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofcharleston.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>866-868-1006</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Charleston SC</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>96</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Charleston SC</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 18:19 UTC (cycle 196)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3849,7 +3849,6 @@
           <t>https://www.metalroofcharleston.com/</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>moreinfo@metalroofcharleston.com</t>
@@ -3879,6 +3878,122 @@
         </is>
       </c>
       <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>RSC Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>rscheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.rscheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Not Working</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>steve.beeler@rscheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(717)299-3914</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Lancaster PA</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lancaster PA</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Nick's Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>callnicksheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://callnicksheatingandcooling.com/birmingham-hvac-contractor/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>info@callnicksheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(205) 736-7049</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>90</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>HVAC contractor Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 18:26 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3964,7 +3964,6 @@
           <t>https://callnicksheatingandcooling.com/birmingham-hvac-contractor/</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>info@callnicksheatingandcooling.com</t>
@@ -3994,6 +3993,66 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Infinite Roofing GC LLC</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>infiniteroofing.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://infiniteroofing.com/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Schedule Your</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>info@infiniteroofinggcllc.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>469-300-5400</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>100</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>roofer Plano TX</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 19:38 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4058,6 +4058,66 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Roof Replacement &amp; Repair in Federal Way, WA</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>redravenexteriors.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.redravenexteriors.com/roofing/federal-way</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Snohomish Co</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>corbin@redravenexteriors.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(425) 375-4360</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>90</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>roof replacement Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 19:39 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4118,6 +4118,62 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Breylin Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>breylinhvac.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://breylinhvac.com/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>breylin06@aol.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>856-718-2786</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Camden NJ</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>80</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>heating and cooling company Camden NJ</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 19:41 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4139,7 +4139,6 @@
           <t>https://breylinhvac.com/</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>breylin06@aol.com</t>
@@ -4169,6 +4168,122 @@
         </is>
       </c>
       <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>247 Bronx Plumbing NYC</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>247bronxplumbingnyc.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://247bronxplumbingnyc.com/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>247bronxplumbingnyc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>347-377-2564</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Bronx NY</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>100</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>plumbing company Bronx NY</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Olympia HVAC Repair, Heating &amp; AC | Perfect Temp Inc</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>perfecttempinc.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://perfecttempinc.com/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Save Money</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>hvac@perfecttempinc.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(360) 890-4312</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Olympia WA</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>90</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>heating and cooling company Olympia WA</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 19:45 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4194,7 +4194,6 @@
           <t>https://247bronxplumbingnyc.com/</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>247bronxplumbingnyc@gmail.com</t>
@@ -4284,6 +4283,126 @@
         </is>
       </c>
       <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>HVACBros Air Conditioning Repair</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>hvacbros.net</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://hvacbros.net/hvac-in-miramar-fl/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Fernando Mendez</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>info@hvacbros.net</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(645) 219-1623</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>90</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>HVAC contractor Miramar FL</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Emcac</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>excelmechanicalcontractors.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://excelmechanicalcontractors.com/miramar/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>salesandservice@emcairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(561) 331-6500</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>90</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>HVAC contractor Miramar FL</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 19:47 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4408,6 +4408,66 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Plumber Elite of Brownsville</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>plumberelitebrownsville.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://plumberelitebrownsville.com/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Direct Infrastructure</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>info@plumberelitebrownsville.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(956) 815-3296</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Brownsville TX</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>90</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>plumber Brownsville TX</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 19:48 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4468,6 +4468,66 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>PSP Trenchless</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>psptrenchless.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.psptrenchless.com/alexandria-va/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Repair We</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>info@psptrenchless.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(703) 343-0767</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Alexandria VA</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>90</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>sewer repair Alexandria VA</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 19:58 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4528,6 +4528,126 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Whitlock Roofing</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>whitlocknm.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://whitlocknm.com/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Whitlock Enterprises</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>admin@whitlocknm.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(505) 890-3488</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>98</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>roof repair company Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>New View Roofing</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>newviewroofing.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://newviewroofing.com/mckinney-tx-roofing-contractor/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>North Dallas</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>info@newviewroofing.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>(469) 425-8232</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>90</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>roofing contractor McKinney TX</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:01 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4648,6 +4648,114 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Plumber  in Roswell, GA | Superior Plumbing</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>plumbersroswellga.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://www.plumbersroswellga.com/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>customerservice@superiorplumbing.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Roswell GA</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>86</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>plumber Roswell GA</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Shield Multiservices</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>shieldmultiservices.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://shieldmultiservices.com/metal-roofing-brownsville-tx</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>shieldmultiservicesrgv@gmail.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(956) 622-6601</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Brownsville TX</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>82</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Brownsville TX</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:20 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4669,13 +4669,11 @@
           <t>https://www.plumbersroswellga.com/</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>customerservice@superiorplumbing.com</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>Roswell GA</t>
@@ -4721,7 +4719,6 @@
           <t>https://shieldmultiservices.com/metal-roofing-brownsville-tx</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>shieldmultiservicesrgv@gmail.com</t>
@@ -4751,6 +4748,66 @@
         </is>
       </c>
       <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Bryan General Contractor LLC</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>bryangeneralcontractorllc.us</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://bryangeneralcontractorllc.us/annapolis-md/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>bryangeneralcontractorllc2025@gmail.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>(240) 286-1720</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>100</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>roof replacement Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:26 UTC (cycle 36)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4813,6 +4813,66 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Rio Rancho, NM | Blue Bear Roofing</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>bluebearroofing.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.bluebearroofing.com/roofing-services-in-rio-rancho-nm</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Blue Bear</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>info@bluebearroofing.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(505) 219-2400</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Rio Rancho NM</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>90</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>roofing contractor Rio Rancho NM</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:34 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4873,6 +4873,66 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Carolina Restoration Pro — Concord NC Roofing, Siding &amp; Gutters</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>carolinarestorationpro.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://carolinarestorationpro.com/concord</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Concord Parkway</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>info@carolinarestorationpro.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(704) 953-2887</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>90</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>roofing contractor Concord NC</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:37 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4933,6 +4933,66 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>fortworthplumber.us</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>fortworthplumber.us</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://fortworthplumber.us/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>More About</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>info@fortworthplumber.us</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>(817) 886-4473</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>90</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>emergency plumber Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:41 UTC (cycle 46)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4993,6 +4993,122 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Casanova Roofing</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>casanovaroofing.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://www.casanovaroofing.com/santa-ana-ca/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>At Casanova</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>john@smith.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(888) 338-0123</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>100</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>roofer Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Bell Heating And Cooling</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>bellhtgandcooling.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>http://www.bellhtgandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>slbell10@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>(812)339-9399</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Bloomington IN</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>56</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bloomington IN</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:48 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5074,7 +5074,6 @@
           <t>http://www.bellhtgandcooling.com/</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>slbell10@yahoo.com</t>
@@ -5104,6 +5103,66 @@
         </is>
       </c>
       <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Jet Heat and Air</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>jetacservice.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://jetacservice.com/ac-installation-little-rock/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Jet Heat</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>brison@jetheatandair.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>501-307-5959</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Little Rock AR</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>90</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>AC installation Little Rock AR</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:53 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5168,6 +5168,66 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Cowtown Drain</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>cowtowndrain.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://cowtowndrain.com/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Drain Customer</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>info@cowtowndrain.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>(817) 674-4085</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>90</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>drain cleaning service Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 20:59 UTC (cycle 58)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5228,6 +5228,66 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Memphis</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>draincleaningmemphis.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://draincleaningmemphis.com/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Robert Washington</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>draincleaningmemphis@gmail.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>(901) 699-0555</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Memphis TN</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>90</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>drain cleaning service Memphis TN</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:00 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5288,6 +5288,66 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>5Star Plumbing Express</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>5starplumbingexpressusa.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://5starplumbingexpressusa.com/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Jobs Completed</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>info@5starplumbingexpressusa.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(831) 279-1447</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>90</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>plumbing company Salinas CA</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:16 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5348,6 +5348,66 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Alba Pro Construction</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>albaproroofing.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://albaproroofing.com/areas/elizabeth</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Services Decks</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>info@albaproroofing.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(201) 994-8577</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Elizabeth NJ</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>roof replacement Elizabeth NJ</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:21 UTC (cycle 73)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5408,6 +5408,62 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Johnson Plumbing, Inc. | Plumbing Repairs | Lawrence, KS</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>johnsonplumbinglawrence.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.johnsonplumbinglawrence.com/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>kpjohnsonplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>785-841-6611</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Lawrence KS</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>84</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>plumber Lawrence KS</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:25 UTC (cycle 76)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5429,7 +5429,6 @@
           <t>https://www.johnsonplumbinglawrence.com/</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>kpjohnsonplumbing@gmail.com</t>
@@ -5459,6 +5458,62 @@
         </is>
       </c>
       <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Roofer | Jacksonville, FL | Ron Russell Roofing</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ronrussellroofing.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.ronrussellroofing.com/</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>ronrussellroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(904) 714-1907</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>90</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>roofer Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:31 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5484,7 +5484,6 @@
           <t>https://www.ronrussellroofing.com/</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>ronrussellroofing@gmail.com</t>
@@ -5514,6 +5513,66 @@
         </is>
       </c>
       <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Province Roofing &amp; Construction -</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>provinceroofingconstruction.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://provinceroofingconstruction.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Competitive Pricing</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>roland@provinceroofingconstruction.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(910) 800-1935</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>100</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>residential roofing company Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:34 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5578,6 +5578,62 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Residential &amp; Commercial Plumbing</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>morelliplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.morelliplumbingllc.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>morelliplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>585-703-1006</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>90</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>plumbing company Rochester NY</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:37 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5599,7 +5599,6 @@
           <t>https://www.morelliplumbingllc.com/</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>morelliplumbing@yahoo.com</t>
@@ -5629,6 +5628,66 @@
         </is>
       </c>
       <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Azerplumb</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>azerplumb.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://azerplumb.com/plumber-alpharetta-ga/</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Alpharetta Whether</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>azerplumb@gmail.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>678-750-2300</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>100</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>plumber Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:42 UTC (cycle 87)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5693,6 +5693,66 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Sprauer Roofing</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>sprauerroofingco.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://www.sprauerroofingco.com/round-rock-roofing/</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>You Found</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>billsprauerroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>737-703-6290</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>90</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>roofer Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:43 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5753,6 +5753,62 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Timber Ridge Plumbing &amp; Heating | Bismarck, ND</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>timberridgephnd.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://www.timberridgephnd.com/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>timberridgeplbg@midconetwork.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>(701) 289-3106</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Bismarck ND</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>100</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>plumber Bismarck ND</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:45 UTC (cycle 89)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5774,7 +5774,6 @@
           <t>https://www.timberridgephnd.com/</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>timberridgeplbg@midconetwork.com</t>
@@ -5804,6 +5803,66 @@
         </is>
       </c>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Plumbing Services | Arlington, TX | Complete Plumbing</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>completeplumbsolutions.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.completeplumbsolutions.com/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Complete Plumbing</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>admin@completeplumbsolutions.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(817) 472-5479</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Arlington TX</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>84</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>plumbing company Arlington TX</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:52 UTC (cycle 94)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5868,6 +5868,66 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Davis Construction &amp; Roofing Co.</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>davisconstructionroofingco.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.davisconstructionroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>South Carolina</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>ddavis@davisconstructionroofingco.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>762-477-3858</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Augusta GA</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>90</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>roofing contractor Augusta GA</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:54 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5928,6 +5928,66 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>J Paul Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>jpaulroofing.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://jpaulroofing.com/roofing-contractors-richardson/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Why Richardson</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>service@jpaulcs.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>469-562-1990</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>100</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>roofing contractor Richardson TX</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 21:55 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5988,6 +5988,66 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Roofing Systems of Hampton Roads</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>roofinghr.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.roofinghr.com/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Why Chesapeake</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>info@roofinghr.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(757) 600-6747</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>90</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>roofing contractor Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:00 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6048,6 +6048,122 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Murfreesboro, TN</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>murfreesborotnroofing.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://murfreesborotnroofing.com/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>bloomingdaleproductions@gmail.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(615) 570-4251</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>100</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>roofing contractor Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Branch Roofing</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>branchroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://branchroofingllc.com/murfreesboro-tn-roofing/</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Owners Brandon</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>info@branchroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>615-931-2756</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>90</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>roofing contractor Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:05 UTC (cycle 103)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6069,7 +6069,6 @@
           <t>https://murfreesborotnroofing.com/</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>bloomingdaleproductions@gmail.com</t>
@@ -6159,6 +6158,126 @@
         </is>
       </c>
       <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Creative Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>creativeheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://creativeheatingcooling.com/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Photo Lupe</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>info@creativeheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>(661) 345-6450</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>90</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Alvarado Roofing, Inc.</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>alvaradoroofing.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://alvaradoroofing.com/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Alvarado Roofing</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>service@alvaradoroofing.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(505) 842-7663</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>80</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>roofing contractor Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:10 UTC (cycle 106)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6283,6 +6283,66 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Christian Brothers Roofing</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>christianbroroofing.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.christianbroroofing.com/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Better Business</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>info@christianbroroofing.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(502) 244-0208</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>100</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>roof replacement Louisville KY</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:14 UTC (cycle 109)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6343,6 +6343,66 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Acosta Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>acostaplumbingfl.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.acostaplumbingfl.com/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Condo Boards</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>acostaplumbingservice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>(305) 634-6676</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>100</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>water heater repair Miami FL</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:26 UTC (cycle 117)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6403,6 +6403,122 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Cruz Plumbing &amp; Rooter Services</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>cruzplumbingandrooter.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.cruzplumbingandrooter.com/fontana</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Cruz Plumbing</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>service@cruzplumbingandrooter.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>833) 453-2731</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Fontana CA</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>90</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>plumbing company Fontana CA</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>American Made Plumbing</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>americanmadeplumbing.co</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://americanmadeplumbing.co/service-area/fontana-ca/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>americanmadeplumb@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(657) 632-8881</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Fontana CA</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>90</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>plumbing company Fontana CA</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:31 UTC (cycle 120)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6484,7 +6484,6 @@
           <t>https://americanmadeplumbing.co/service-area/fontana-ca/</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>americanmadeplumb@yahoo.com</t>
@@ -6514,6 +6513,62 @@
         </is>
       </c>
       <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>TC HVAC Services</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>tchvacservices.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://tchvacservices.com/arlington-va-hvac/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>info@tchvacservices.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>703-721-4770</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Arlington VA</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>100</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>heating and cooling company Arlington VA</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:32 UTC (cycle 121)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6539,7 +6539,6 @@
           <t>https://tchvacservices.com/arlington-va-hvac/</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>info@tchvacservices.com</t>
@@ -6569,6 +6568,62 @@
         </is>
       </c>
       <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Tropic Air Conditioning Inc.</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>tropicairfl.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://tropicairfl.com/air-conditioning-installation/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>tropicair1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>(941) 751-2653</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>90</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>AC installation Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:35 UTC (cycle 123)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6594,7 +6594,6 @@
           <t>https://tropicairfl.com/air-conditioning-installation/</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>tropicair1@gmail.com</t>
@@ -6624,6 +6623,66 @@
         </is>
       </c>
       <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>TMS Quality Metal Roofing | Metal Roofing in San Antonio, TX</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>tmsqualitymetalroofing.net</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://tmsqualitymetalroofing.net/</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Top Rated</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>tmsqualityroof@gmail.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(210) 772-0833</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>90</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>metal roofing contractor San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:37 UTC (cycle 124)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6688,6 +6688,238 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Pipeline Plumbing, Inc - Tallahassee Big Bend</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>pipelineplumbingusa.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://pipelineplumbingusa.com/</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>lemonad@jovanny.ru</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>850-738-7473</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>90</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>plumbing company Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Home | Watts Cooling, Heating &amp; Plumbing, LLC</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>wattshvacplumbing.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.wattshvacplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Carre Welsh</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>info@bluecollar.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>(850) 224-4822</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>88</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>plumbing company Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Cureton Plumbing</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>curetonplumbing.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://curetonplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>info@curetonplumbing.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>850-222-4412</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>88</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>plumbing company Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>JBP</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>jimbennettsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.jimbennettsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Jim Bennett</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>dispatch@jimbennetts.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>850-878-3178</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>72</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>plumbing company Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:51 UTC (cycle 134)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6709,7 +6709,6 @@
           <t>https://pipelineplumbingusa.com/</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>lemonad@jovanny.ru</t>
@@ -6825,7 +6824,6 @@
           <t>https://curetonplumbing.com/</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>info@curetonplumbing.com</t>
@@ -6915,6 +6913,62 @@
         </is>
       </c>
       <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Dial Plumbing</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>dialplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://dialplumbingservice.com/mount-pleasant-sc-plumber</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>lemonad@jovanny.ru</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>(843) 475-8391</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Mount Pleasant SC</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>90</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>plumber Mount Pleasant SC</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 22:53 UTC (cycle 135)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6939,7 +6939,6 @@
           <t>https://dialplumbingservice.com/mount-pleasant-sc-plumber</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>lemonad@jovanny.ru</t>
@@ -6969,6 +6968,66 @@
         </is>
       </c>
       <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Liberty Drain</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>libertydrain.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://libertydrain.com/service-area/mount-vernon/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Liberty Drain</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>tj@libertydrain.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(888) 578-2240</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>84</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>drain cleaning service Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:10 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7033,6 +7033,126 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Furnace Repair Sacramento | Capital City Comfort</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>capitalcitycomfort.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://capitalcitycomfort.com/furnace-repair-sacramento</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Clear Communication</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>capitalcitycomfort@att.net</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>(916) 390-0025</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Sacramento CA</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>90</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>furnace repair Sacramento CA</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Kaliber Roofing</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>kaliberroofing.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://kaliberroofing.com/rock-hill-sc/</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Local Roofing</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>support@kaliberroofing.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(980) 414-3038</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>90</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>roofer Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:12 UTC (cycle 148)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7153,6 +7153,122 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Red Rock Roofing</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>redrockroofing.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://redrockroofing.com/arvada-roofing-company/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Served What</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>info@redrockroofing.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>720-735-7663</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Arvada CO</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>100</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>roof repair company Arvada CO</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>mgeneral-construction.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://mgeneral-construction.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>m.general.const@gmail.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>347-665-8493</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>90</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Queens NY</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:18 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7234,7 +7234,6 @@
           <t>https://mgeneral-construction.com/metal-roofing/</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>m.general.const@gmail.com</t>
@@ -7264,6 +7263,62 @@
         </is>
       </c>
       <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Hillsboro, OR 97123</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>hillsborodraincleaning.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://hillsborodraincleaning.com/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>admin@pinkflamingoplumbingco.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>(503) 389-3716</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>88</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>drain cleaning service Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:30 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7289,7 +7289,6 @@
           <t>https://hillsborodraincleaning.com/</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>admin@pinkflamingoplumbingco.com</t>
@@ -7319,6 +7318,66 @@
         </is>
       </c>
       <c r="L118" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Roof MD</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>roof-md.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://www.roof-md.com/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Murfreesboro Verified</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>office@roof-md.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>615-678-2646</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>100</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>roof replacement Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:31 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7383,6 +7383,62 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Report a Sewer Problem</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>norfolk.gov</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.norfolk.gov/636/Wastewater</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>testold@domain.org</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>757-823-1000</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Norfolk VA</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>100</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>sewer repair Norfolk VA</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:36 UTC (cycle 164)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7404,7 +7404,6 @@
           <t>https://www.norfolk.gov/636/Wastewater</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
           <t>testold@domain.org</t>
@@ -7434,6 +7433,66 @@
         </is>
       </c>
       <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Residential Roofing in Roanoke, VA | Cook  S&amp;W Co.</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>cooksiding.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.cooksiding.com/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Customer Satisfaction</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>info@cooksiding.com</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(540) 389-6104</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Roanoke VA</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>residential roofing company Roanoke VA</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:37 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7498,6 +7498,66 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Stockton, CA Plumber</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>stocktoncaplumbing.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://stocktoncaplumbing.com/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Signs You</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>hello@stocktoncaplumbing.com</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>209 444 1473</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>76</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>drain cleaning service Stockton CA</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:45 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7558,6 +7558,66 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Texas Roofing Austin</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>texasroofingaustin.com</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://texasroofingaustin.com/</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Expert Craftsmanship</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>info@texasroofingaustin.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(512) 773-6066</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>90</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>roofing contractor Austin TX</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:56 UTC (cycle 178)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7618,6 +7618,66 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Almco Plumbing</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>almcoplumbing.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://almcoplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Sewer Trenchless</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>office@almcoplumbing.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>(858) 544-6331</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>100</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>plumbing company San Diego CA</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-23 23:59 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-23.xlsx
+++ b/output/leads_2026-09-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7678,6 +7678,66 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Integrity Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>ctintegrity.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://ctintegrity.com/roofing/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Owner Sergio</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>sergio@ctintegrity.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>(860) 359-1569</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Hartford CT</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>90</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>roof replacement Hartford CT</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>